<commit_message>
fix: ajuste Familia Guzman Moreno a 4 pases y Alexis Rubiano a 1 pase individual
</commit_message>
<xml_diff>
--- a/Lista_Invitados_y_Pases_Boda.xlsx
+++ b/Lista_Invitados_y_Pases_Boda.xlsx
@@ -570,7 +570,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>📊 Total de Invitaciones (Mensajes): 52   |   👥 Total de Pases / Personas Estimadas: 93 pases</t>
+          <t>📊 Total de Invitaciones (Mensajes): 52   |   👥 Total de Pases / Personas Estimadas: 91 pases</t>
         </is>
       </c>
     </row>
@@ -1322,11 +1322,11 @@
         </is>
       </c>
       <c r="D30" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Familia (5)</t>
+          <t>Familia (4)</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Alexis Rubiano &amp; Sra</t>
+          <t>Alexis Rubiano</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -1910,16 +1910,16 @@
         </is>
       </c>
       <c r="D51" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Pareja</t>
+          <t>Individual</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=alexis-rubiano-y-sra</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=alexis-rubiano</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="E57" s="14" t="inlineStr">
         <is>
-          <t>93 Personas</t>
+          <t>91 Personas</t>
         </is>
       </c>
       <c r="F57" s="12" t="n"/>

</xml_diff>

<commit_message>
feat: lista definitiva oficial de 49 invitados y 85 pases segun especificacion final de los novios
</commit_message>
<xml_diff>
--- a/Lista_Invitados_y_Pases_Boda.xlsx
+++ b/Lista_Invitados_y_Pases_Boda.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -570,7 +570,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>📊 Total de Invitaciones (Mensajes): 52   |   👥 Total de Pases / Personas Estimadas: 91 pases</t>
+          <t>📊 Total de Invitaciones (Mensajes): 49   |   👥 Total de Pases / Personas Estimadas: 85 pases</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Luisa y Fercho</t>
+          <t>Oscar y Blanca</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>3172959658</t>
+          <t>3178492983</t>
         </is>
       </c>
       <c r="D39" s="6" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=luisa-y-fercho</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=oscar-y-blanca</t>
         </is>
       </c>
     </row>
@@ -1593,25 +1593,25 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Fercho y Luisa</t>
+          <t>Maria Jose</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>3178411896</t>
+          <t>3187026437</t>
         </is>
       </c>
       <c r="D40" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Pareja</t>
+          <t>Individual</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=fercho-y-luisa</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=maria-jose</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1621,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Oscar y Blanca</t>
+          <t>Luis y Julieth</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>3178492983</t>
+          <t>3204545796</t>
         </is>
       </c>
       <c r="D41" s="6" t="n">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=oscar-y-blanca</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=luis-y-julieth</t>
         </is>
       </c>
     </row>
@@ -1649,25 +1649,25 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Maria Jose</t>
+          <t>Fernando y Alejandra</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>3187026437</t>
+          <t>3205582770</t>
         </is>
       </c>
       <c r="D42" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>Pareja</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=maria-jose</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=fernando-y-alejandra</t>
         </is>
       </c>
     </row>
@@ -1677,12 +1677,12 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Luis y Julieth</t>
+          <t>Yesid y Martha</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>3204545796</t>
+          <t>3205633432</t>
         </is>
       </c>
       <c r="D43" s="6" t="n">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=luis-y-julieth</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=yesid-y-martha</t>
         </is>
       </c>
     </row>
@@ -1705,12 +1705,12 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Fernando y Alejandra</t>
+          <t>Santiago y Valen</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>3205582770</t>
+          <t>3212082769</t>
         </is>
       </c>
       <c r="D44" s="10" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=fernando-y-alejandra</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=santiago-y-valen</t>
         </is>
       </c>
     </row>
@@ -1733,12 +1733,12 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Yesid y Martha</t>
+          <t>Camilo y Lina</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>3205633432</t>
+          <t>3212318833</t>
         </is>
       </c>
       <c r="D45" s="6" t="n">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=yesid-y-martha</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=camilo-y-lina</t>
         </is>
       </c>
     </row>
@@ -1761,25 +1761,25 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Santiago y Valen</t>
+          <t>Familia Galindo Moreno</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>3212082769</t>
+          <t>3213221773</t>
         </is>
       </c>
       <c r="D46" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>Pareja</t>
+          <t>Familia (3)</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=santiago-y-valen</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=familia-galindo-moreno</t>
         </is>
       </c>
     </row>
@@ -1789,25 +1789,25 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Camilo y Lina</t>
+          <t>Familia Moreno Gonzalez</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>3212318833</t>
+          <t>3222307829</t>
         </is>
       </c>
       <c r="D47" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Pareja</t>
+          <t>Familia (4)</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=camilo-y-lina</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=familia-moreno-gonzalez</t>
         </is>
       </c>
     </row>
@@ -1817,25 +1817,25 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Familia Galindo Moreno</t>
+          <t>Victor y Xilenia</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>3213221773</t>
+          <t>3228452238</t>
         </is>
       </c>
       <c r="D48" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>Familia (3)</t>
+          <t>Pareja</t>
         </is>
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=familia-galindo-moreno</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=victor-y-xilenia</t>
         </is>
       </c>
     </row>
@@ -1845,25 +1845,25 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Familia Moreno Gonzalez</t>
+          <t>Alexis Rubiano &amp; Sra</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>3222307829</t>
+          <t>3148942652</t>
         </is>
       </c>
       <c r="D49" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Familia (4)</t>
+          <t>Individual</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=familia-moreno-gonzalez</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=alexis-rubiano-y-sra</t>
         </is>
       </c>
     </row>
@@ -1873,12 +1873,12 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Victor y Xilenia</t>
+          <t>Javier &amp; Sra</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>3228452238</t>
+          <t>3045963615</t>
         </is>
       </c>
       <c r="D50" s="10" t="n">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=victor-y-xilenia</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=javier-y-sra</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1901,12 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Alexis Rubiano</t>
+          <t>Yeison</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>3148942652</t>
+          <t>3154383970</t>
         </is>
       </c>
       <c r="D51" s="6" t="n">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=alexis-rubiano</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=yeison</t>
         </is>
       </c>
     </row>
@@ -1929,25 +1929,25 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Javier &amp; Sra</t>
+          <t>Daniela</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>3045963615</t>
+          <t>3175844709</t>
         </is>
       </c>
       <c r="D52" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>Pareja</t>
+          <t>Individual</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=javier-y-sra</t>
+          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=daniela</t>
         </is>
       </c>
     </row>
@@ -1957,12 +1957,12 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Yeison</t>
+          <t>Juan Pablo</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>3154383970</t>
+          <t>3178688336</t>
         </is>
       </c>
       <c r="D53" s="6" t="n">
@@ -1975,116 +1975,32 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=yeison</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>Daniela</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>3175844709</t>
-        </is>
-      </c>
-      <c r="D54" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Individual</t>
-        </is>
-      </c>
-      <c r="F54" s="11" t="inlineStr">
-        <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=daniela</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Juan Pablo</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>3178688336</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>Individual</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=juan-pablo</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="8" t="n">
-        <v>52</v>
-      </c>
-      <c r="B56" s="9" t="inlineStr">
-        <is>
-          <t>Prueba Luisa</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>3172959658</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F56" s="11" t="inlineStr">
-        <is>
-          <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=prueba-luisa</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="26" customHeight="1">
-      <c r="A57" s="12" t="inlineStr"/>
-      <c r="B57" s="13" t="inlineStr">
+    <row r="54" ht="26" customHeight="1">
+      <c r="A54" s="12" t="inlineStr"/>
+      <c r="B54" s="13" t="inlineStr">
         <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="C57" s="14" t="inlineStr">
-        <is>
-          <t>52 Números</t>
-        </is>
-      </c>
-      <c r="D57" s="15">
-        <f>SUM(D5:D56)</f>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>49 Números</t>
+        </is>
+      </c>
+      <c r="D54" s="15">
+        <f>SUM(D5:D53)</f>
         <v/>
       </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>91 Personas</t>
-        </is>
-      </c>
-      <c r="F57" s="12" t="n"/>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>85 Personas</t>
+        </is>
+      </c>
+      <c r="F54" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2141,9 +2057,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: integrar supabase cloud database, sincronizacion en tiempo real y 27 confirmados oficiales
</commit_message>
<xml_diff>
--- a/Lista_Invitados_y_Pases_Boda.xlsx
+++ b/Lista_Invitados_y_Pases_Boda.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,9 +50,20 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <color rgb="00EF6C00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <color rgb="002E5B82"/>
       <sz val="9"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -66,8 +77,14 @@
       <color rgb="008F6E2B"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002C3821"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -94,8 +111,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+        <bgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F9FAF8"/>
         <bgColor rgb="00F9FAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -139,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -159,29 +188,38 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -549,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -557,7 +595,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -570,7 +609,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>📊 Total de Invitaciones (Mensajes): 50   |   👥 Total de Pases / Personas Estimadas: 88 pases</t>
+          <t>📊 Total: 50 Inv (88 pases)   |   ✅ Confirmados: 27 Inv (49 pases)   |   ⏳ Pendientes: 23 Inv (39 pases)</t>
         </is>
       </c>
     </row>
@@ -603,6 +642,11 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
+          <t>Estado RSVP</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
           <t>Enlace Tarjeta Interactiva</t>
         </is>
       </c>
@@ -631,33 +675,43 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=german-y-mary</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Angela y Gaby</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>3102227404</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="D6" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=angela-y-gaby</t>
         </is>
@@ -687,33 +741,43 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=argenis</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Luis y Sandra</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>3006517876</t>
         </is>
       </c>
-      <c r="D8" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="D8" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=luis-y-sandra</t>
         </is>
@@ -743,33 +807,43 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=juan-y-paola</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Jorge y Alejandra</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>3134750682</t>
         </is>
       </c>
-      <c r="D10" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="D10" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=jorge-y-alejandra</t>
         </is>
@@ -799,33 +873,43 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=enrique-y-anita</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Alejo y Kelly</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>3143119452</t>
         </is>
       </c>
-      <c r="D12" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="D12" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=alejo-y-kelly</t>
         </is>
@@ -855,33 +939,43 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=wilson</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Ferenc y Diana</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>3153148043</t>
         </is>
       </c>
-      <c r="D14" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="D14" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=ferenc-y-diana</t>
         </is>
@@ -911,33 +1005,43 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=daniel</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="8" t="n">
+      <c r="A16" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Fabian Moreno</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>3174409887</t>
         </is>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=fabian-moreno</t>
         </is>
@@ -967,33 +1071,43 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=johnatan-y-natalie</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="8" t="n">
+      <c r="A18" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Yeisson y Lorena</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>3214900317</t>
         </is>
       </c>
-      <c r="D18" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
+      <c r="D18" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=yeisson-y-lorena</t>
         </is>
@@ -1023,33 +1137,43 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=marcela</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="8" t="n">
+      <c r="A20" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Katalina</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>3161958838</t>
         </is>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=katalina</t>
         </is>
@@ -1077,35 +1201,45 @@
           <t>Individual</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=norma</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="8" t="n">
+      <c r="A22" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>Xiomara</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>3106959140</t>
         </is>
       </c>
-      <c r="D22" s="10" t="n">
+      <c r="D22" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="F22" s="11" t="inlineStr">
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=xiomara</t>
         </is>
@@ -1135,33 +1269,43 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=andrea</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="8" t="n">
+      <c r="A24" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Nubia</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>3123962885</t>
         </is>
       </c>
-      <c r="D24" s="10" t="n">
+      <c r="D24" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="F24" s="11" t="inlineStr">
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=nubia</t>
         </is>
@@ -1191,33 +1335,43 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=jairo-e-irma</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="8" t="n">
+      <c r="A26" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Oscar y Lina</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>3168258737</t>
         </is>
       </c>
-      <c r="D26" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr">
+      <c r="D26" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=oscar-y-lina</t>
         </is>
@@ -1247,33 +1401,43 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=martha-diaz</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="8" t="n">
+      <c r="A28" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Ciro y Adriana</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>3162543924</t>
         </is>
       </c>
-      <c r="D28" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="inlineStr">
+      <c r="D28" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=ciro-y-adriana</t>
         </is>
@@ -1303,33 +1467,43 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=miryam</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="8" t="n">
+      <c r="A30" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Familia Guzman Moreno</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>3176999226</t>
         </is>
       </c>
-      <c r="D30" s="10" t="n">
+      <c r="D30" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>Familia (5)</t>
         </is>
       </c>
-      <c r="F30" s="11" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=familia-guzman-moreno</t>
         </is>
@@ -1357,35 +1531,45 @@
           <t>Individual</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=camilo</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="8" t="n">
+      <c r="A32" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>Mayra</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>3118965505</t>
         </is>
       </c>
-      <c r="D32" s="10" t="n">
+      <c r="D32" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="F32" s="11" t="inlineStr">
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=mayra</t>
         </is>
@@ -1413,35 +1597,45 @@
           <t>Individual</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=leidy</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="8" t="n">
+      <c r="A34" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Raul y Sandra</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>3015092937</t>
         </is>
       </c>
-      <c r="D34" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F34" s="11" t="inlineStr">
+      <c r="D34" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=raul-y-sandra</t>
         </is>
@@ -1469,35 +1663,45 @@
           <t>Pareja</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=liss-y-vivi</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="8" t="n">
+      <c r="A36" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Familia Orozco Moreno</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>3046808114</t>
         </is>
       </c>
-      <c r="D36" s="10" t="n">
+      <c r="D36" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E36" s="9" t="inlineStr">
         <is>
           <t>Familia (4)</t>
         </is>
       </c>
-      <c r="F36" s="11" t="inlineStr">
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=familia-orozco-moreno</t>
         </is>
@@ -1527,33 +1731,43 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=alberto-y-edith</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="8" t="n">
+      <c r="A38" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Jairo y Diana</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>3134699155</t>
         </is>
       </c>
-      <c r="D38" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F38" s="11" t="inlineStr">
+      <c r="D38" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=jairo-y-diana</t>
         </is>
@@ -1581,35 +1795,45 @@
           <t>Pareja</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=oscar-y-blanca</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="8" t="n">
+      <c r="A40" s="9" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>Maria Jose</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>3187026437</t>
         </is>
       </c>
-      <c r="D40" s="10" t="n">
+      <c r="D40" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="F40" s="11" t="inlineStr">
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=maria-jose</t>
         </is>
@@ -1637,35 +1861,45 @@
           <t>Pareja</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=luis-y-julieth</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="8" t="n">
+      <c r="A42" s="9" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Fernando y Alejandra</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>3205582770</t>
         </is>
       </c>
-      <c r="D42" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F42" s="11" t="inlineStr">
+      <c r="D42" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=fernando-y-alejandra</t>
         </is>
@@ -1693,35 +1927,45 @@
           <t>Pareja</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
+      <c r="F43" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=yesid-y-martha</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="8" t="n">
+      <c r="A44" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>Santiago y Valen</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>3212082769</t>
         </is>
       </c>
-      <c r="D44" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F44" s="11" t="inlineStr">
+      <c r="D44" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G44" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=santiago-y-valen</t>
         </is>
@@ -1749,35 +1993,45 @@
           <t>Pareja</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F45" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=camilo-y-lina</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="8" t="n">
+      <c r="A46" s="9" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>Familia Galindo Moreno</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>3213221773</t>
         </is>
       </c>
-      <c r="D46" s="10" t="n">
+      <c r="D46" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E46" s="9" t="inlineStr">
         <is>
           <t>Familia (3)</t>
         </is>
       </c>
-      <c r="F46" s="11" t="inlineStr">
+      <c r="F46" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G46" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=familia-galindo-moreno</t>
         </is>
@@ -1805,35 +2059,45 @@
           <t>Familia (4)</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F47" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=familia-moreno-gonzalez</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="8" t="n">
+      <c r="A48" s="9" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B48" s="10" t="inlineStr">
         <is>
           <t>Victor y Xilenia</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>3228452238</t>
         </is>
       </c>
-      <c r="D48" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F48" s="11" t="inlineStr">
+      <c r="D48" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G48" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=victor-y-xilenia</t>
         </is>
@@ -1863,33 +2127,43 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=alexis-rubiano-y-sra</t>
         </is>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="8" t="n">
+      <c r="A50" s="9" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>Javier &amp; Sra</t>
         </is>
       </c>
-      <c r="C50" s="8" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>3045963615</t>
         </is>
       </c>
-      <c r="D50" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F50" s="11" t="inlineStr">
+      <c r="D50" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G50" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=javier-y-sra</t>
         </is>
@@ -1917,35 +2191,45 @@
           <t>Individual</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
+      <c r="F51" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=yeison</t>
         </is>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="8" t="n">
+      <c r="A52" s="9" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="9" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>Daniela</t>
         </is>
       </c>
-      <c r="C52" s="8" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>3175844709</t>
         </is>
       </c>
-      <c r="D52" s="10" t="n">
+      <c r="D52" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E52" s="8" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="F52" s="11" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G52" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=daniela</t>
         </is>
@@ -1973,119 +2257,134 @@
           <t>Individual</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
+      <c r="F53" s="13" t="inlineStr">
+        <is>
+          <t>✅ Confirmado</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=juan-pablo</t>
         </is>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="8" t="n">
+      <c r="A54" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="9" t="inlineStr">
+      <c r="B54" s="10" t="inlineStr">
         <is>
           <t>Julian y Camila</t>
         </is>
       </c>
-      <c r="C54" s="8" t="inlineStr">
+      <c r="C54" s="9" t="inlineStr">
         <is>
           <t>3125304333</t>
         </is>
       </c>
-      <c r="D54" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Pareja</t>
-        </is>
-      </c>
-      <c r="F54" s="11" t="inlineStr">
+      <c r="D54" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>⏳ Pendiente</t>
+        </is>
+      </c>
+      <c r="G54" s="12" t="inlineStr">
         <is>
           <t>https://boda-fernando-luisa.vercel.app/index.html?invitado=julian-y-camila</t>
         </is>
       </c>
     </row>
     <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="12" t="inlineStr"/>
-      <c r="B55" s="13" t="inlineStr">
+      <c r="A55" s="14" t="inlineStr"/>
+      <c r="B55" s="15" t="inlineStr">
         <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="C55" s="14" t="inlineStr">
+      <c r="C55" s="16" t="inlineStr">
         <is>
           <t>50 Números</t>
         </is>
       </c>
-      <c r="D55" s="15">
+      <c r="D55" s="17">
         <f>SUM(D5:D54)</f>
         <v/>
       </c>
-      <c r="E55" s="14" t="inlineStr">
+      <c r="E55" s="16" t="inlineStr">
         <is>
           <t>88 Personas</t>
         </is>
       </c>
-      <c r="F55" s="12" t="n"/>
+      <c r="F55" s="18" t="inlineStr">
+        <is>
+          <t>27 Conf / 23 Pend</t>
+        </is>
+      </c>
+      <c r="G55" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>